<commit_message>
feat(reviews): 11c review import from Excel — minimal version
Data model: Review gets source, importBatch, materialConnection (default none).
Template: docs/reviews/import-template.xlsx with five-line EN+ZH README.
Importer: scripts/import-reviews.mjs validates all rows, de-dups, dry-run.
Display: connection line only for non-none values; no split counts.
Policy: one paragraph replacing the numbered list; removal rules kept.
HOW_REVIEWS_WORK: single constant, short form removed.
API: source: 'order' added to invite-based submissions.
Tests: validation, de-dup, dry-run, connection labels, policy content.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reviews/import-template.xlsx
+++ b/docs/reviews/import-template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>product_handle</t>
   </si>
@@ -38,16 +38,13 @@
     <t>date</t>
   </si>
   <si>
-    <t>language</t>
+    <t>material_connection</t>
   </si>
   <si>
     <t>consent</t>
   </si>
   <si>
-    <t>material_connection</t>
-  </si>
-  <si>
-    <t>source_note</t>
+    <t>note</t>
   </si>
   <si>
     <t>charuco-composite-a3</t>
@@ -71,127 +68,46 @@
     <t>2026-09-15</t>
   </si>
   <si>
-    <t>en</t>
+    <t>free_sample</t>
   </si>
   <si>
     <t>yes</t>
   </si>
   <si>
-    <t>free_sample</t>
-  </si>
-  <si>
     <t>Sample sent 2026-08-01; written permission received 2026-09-20 via e-mail</t>
   </si>
   <si>
-    <t>REVIEW IMPORT RULES</t>
+    <t>1. The reviewer used this product.</t>
+  </si>
+  <si>
+    <t>2. Text is published as written.</t>
+  </si>
+  <si>
+    <t>3. Every review received is imported, good or bad.</t>
+  </si>
+  <si>
+    <t>4. Mark free sample / discount / insider in material_connection.</t>
+  </si>
+  <si>
+    <t>5. Keep the permission e-mail on file.</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>=== English ===</t>
-  </si>
-  <si>
-    <t>1. The reviewer must have actually used the product listed in product_handle.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Never reuse a review for a different product.</t>
-  </si>
-  <si>
-    <t>2. Every review received is imported, positive or negative.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Leaving out negative reviews is review suppression and violates FTC guidelines.</t>
-  </si>
-  <si>
-    <t>3. No reward may depend on what the review says.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   You may provide a free sample or discount, but the reviewer must be free to write anything.</t>
-  </si>
-  <si>
-    <t>4. Free samples, discounts, and any employee/relative/insider relationship</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   must be declared in the material_connection column.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - none: reviewer bought the product independently</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - free_sample: reviewer received a free unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - discount: reviewer received a discounted unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - insider: reviewer is an employee, contractor, relative, or has another connection to Calib.Tools</t>
-  </si>
-  <si>
-    <t>5. The review text (body) is the reviewer's own words. Never edit the text.</t>
-  </si>
-  <si>
-    <t>6. consent must be "yes" — you must have written permission on file</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   (e.g. an e-mail) to publish the reviewer's name and text.</t>
-  </si>
-  <si>
-    <t>7. source_note is internal only and never published.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Record where the review came from and the date of the permission e-mail.</t>
-  </si>
-  <si>
-    <t>=== 中文 ===</t>
-  </si>
-  <si>
-    <t>1. 评论者必须实际使用过 product_handle 列中指定的产品。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   不得将一条评论用于另一个产品。</t>
-  </si>
-  <si>
-    <t>2. 收到的每一条评论都必须导入，无论正面还是负面。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   省略负面评论属于评论压制，违反 FTC 规定。</t>
-  </si>
-  <si>
-    <t>3. 任何奖励不得取决于评论内容。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   可以提供免费样品或折扣，但评论者必须可以自由发表任何内容。</t>
-  </si>
-  <si>
-    <t>4. 免费样品、折扣以及任何员工/亲属/关联方关系</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   必须在 material_connection 列中声明。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - none: 评论者独立购买</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - free_sample: 评论者收到了免费样品</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - discount: 评论者收到了折扣</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - insider: 评论者是 Calib.Tools 的员工、承包商、亲属或其他关联方</t>
-  </si>
-  <si>
-    <t>5. 评论正文 (body) 是评论者的原话。不得编辑文本。</t>
-  </si>
-  <si>
-    <t>6. consent 必须填 "yes" —— 必须有书面许可（如邮件）允许发布评论者姓名和文本。</t>
-  </si>
-  <si>
-    <t>7. source_note 仅供内部使用，不会公开发布。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   记录评论来源以及许可邮件的日期。</t>
+    <t>1. 评论者使用过该产品。</t>
+  </si>
+  <si>
+    <t>2. 文本原样发布。</t>
+  </si>
+  <si>
+    <t>3. 收到的每条评论都导入，好坏都要。</t>
+  </si>
+  <si>
+    <t>4. 在 material_connection 中标注免费样品 / 折扣 / 内部人员。</t>
+  </si>
+  <si>
+    <t>5. 保留授权邮件。</t>
   </si>
 </sst>
 </file>
@@ -577,7 +493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -587,12 +503,12 @@
     <col min="5" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="50" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="11" max="11" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -626,46 +542,40 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>12</v>
       </c>
       <c r="B2">
         <v>5</v>
       </c>
       <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>17</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>18</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>20</v>
-      </c>
-      <c r="K2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -674,11 +584,11 @@
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: none, free_sample, discount, insider." sqref="I2:I1000">
+      <formula1>"none,free_sample,discount,insider"</formula1>
+    </dataValidation>
     <dataValidation type="list" showErrorMessage="1" errorTitle="Consent required" error="Consent must be &quot;yes&quot;. Written permission to publish name and text must be on file." sqref="J2:J1000">
       <formula1>"yes"</formula1>
-    </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: none, free_sample, discount, insider." sqref="K2:K1000">
-      <formula1>"none,free_sample,discount,insider"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -688,7 +598,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A53"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
@@ -696,17 +606,17 @@
   <sheetData>
     <row r="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -716,17 +626,17 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
@@ -741,222 +651,12 @@
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>